<commit_message>
feat(repeat): round 3 re-prepares B5 and BIN2 whole, both phases
The user's call: two tubes are cheap, so both phases are re-sampled and the organic
KF re-measured instead of patching the aqueous side only. Entry sheet now 8 vials.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/out/repeat3_entry.xlsx
+++ b/out/repeat3_entry.xlsx
@@ -93,7 +93,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="21">
+  <cellXfs count="20">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -118,7 +118,6 @@
     </xf>
     <xf numFmtId="164" fontId="3" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="2" fontId="3" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="1" fillId="2" borderId="0" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
       <protection locked="0" hidden="0"/>
     </xf>
@@ -201,6 +200,36 @@
     </indexedColors>
   </colors>
 </styleSheet>
+</file>
+
+<file path=xl/comments/comment1.xml><?xml version="1.0" encoding="utf-8"?>
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <authors>
+    <author>make_entry_workbook</author>
+  </authors>
+  <commentList>
+    <comment ref="M9" authorId="0" shapeId="0">
+      <text>
+        <t>Campaign 1: 5.883 %</t>
+      </text>
+    </comment>
+    <comment ref="M10" authorId="0" shapeId="0">
+      <text>
+        <t>Campaign 1: 5.737 %</t>
+      </text>
+    </comment>
+    <comment ref="M13" authorId="0" shapeId="0">
+      <text>
+        <t>Campaign 1: 2.1978 %</t>
+      </text>
+    </comment>
+    <comment ref="M14" authorId="0" shapeId="0">
+      <text>
+        <t>Campaign 1: 2.2258 %</t>
+      </text>
+    </comment>
+  </commentList>
+</comments>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -492,7 +521,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:P12"/>
+  <dimension ref="A1:P16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -827,17 +856,17 @@
       </c>
       <c r="B9" s="11" t="inlineStr">
         <is>
-          <t>B5-B1</t>
+          <t>B5-T1</t>
         </is>
       </c>
       <c r="C9" s="11" t="inlineStr">
         <is>
-          <t>Inferior</t>
+          <t>Superior</t>
         </is>
       </c>
       <c r="D9" s="11" t="inlineStr">
         <is>
-          <t>aqueous</t>
+          <t>organic</t>
         </is>
       </c>
       <c r="E9" s="12" t="n"/>
@@ -862,11 +891,11 @@
         <f>IF(AND(ISNUMBER(J9),ISNUMBER(K9)),IF(J9&gt;0,(J9+K9)/J9,""),"")</f>
         <v/>
       </c>
-      <c r="M9" s="16" t="n"/>
-      <c r="N9" s="16" t="n"/>
+      <c r="M9" s="13" t="n"/>
+      <c r="N9" s="13" t="n"/>
       <c r="O9" s="11" t="inlineStr">
         <is>
-          <t>n/a: by difference</t>
+          <t>fresh: type the new KF</t>
         </is>
       </c>
       <c r="P9" s="13" t="n"/>
@@ -879,111 +908,111 @@
       </c>
       <c r="B10" s="3" t="inlineStr">
         <is>
-          <t>B5-B2</t>
+          <t>B5-T2</t>
         </is>
       </c>
       <c r="C10" s="3" t="inlineStr">
         <is>
-          <t>Inferior</t>
+          <t>Superior</t>
         </is>
       </c>
       <c r="D10" s="3" t="inlineStr">
         <is>
-          <t>aqueous</t>
-        </is>
-      </c>
-      <c r="E10" s="17" t="n"/>
-      <c r="F10" s="18" t="n">
+          <t>organic</t>
+        </is>
+      </c>
+      <c r="E10" s="16" t="n"/>
+      <c r="F10" s="17" t="n">
         <v>300</v>
       </c>
-      <c r="G10" s="17" t="n"/>
+      <c r="G10" s="16" t="n"/>
       <c r="H10" s="3">
         <f>1000-F10</f>
         <v/>
       </c>
-      <c r="I10" s="17" t="n"/>
-      <c r="J10" s="19">
+      <c r="I10" s="16" t="n"/>
+      <c r="J10" s="18">
         <f>IF(AND(ISNUMBER(E10),ISNUMBER(G10)),G10-E10,"")</f>
         <v/>
       </c>
-      <c r="K10" s="19">
+      <c r="K10" s="18">
         <f>IF(AND(ISNUMBER(G10),ISNUMBER(I10)),I10-G10,"")</f>
         <v/>
       </c>
-      <c r="L10" s="20">
+      <c r="L10" s="19">
         <f>IF(AND(ISNUMBER(J10),ISNUMBER(K10)),IF(J10&gt;0,(J10+K10)/J10,""),"")</f>
         <v/>
       </c>
-      <c r="M10" s="5" t="n"/>
-      <c r="N10" s="5" t="n"/>
+      <c r="M10" s="17" t="n"/>
+      <c r="N10" s="17" t="n"/>
       <c r="O10" s="3" t="inlineStr">
         <is>
+          <t>fresh: type the new KF</t>
+        </is>
+      </c>
+      <c r="P10" s="17" t="n"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="3" t="inlineStr">
+        <is>
+          <t>B5</t>
+        </is>
+      </c>
+      <c r="B11" s="3" t="inlineStr">
+        <is>
+          <t>B5-B1</t>
+        </is>
+      </c>
+      <c r="C11" s="3" t="inlineStr">
+        <is>
+          <t>Inferior</t>
+        </is>
+      </c>
+      <c r="D11" s="3" t="inlineStr">
+        <is>
+          <t>aqueous</t>
+        </is>
+      </c>
+      <c r="E11" s="16" t="n"/>
+      <c r="F11" s="17" t="n">
+        <v>300</v>
+      </c>
+      <c r="G11" s="16" t="n"/>
+      <c r="H11" s="3">
+        <f>1000-F11</f>
+        <v/>
+      </c>
+      <c r="I11" s="16" t="n"/>
+      <c r="J11" s="18">
+        <f>IF(AND(ISNUMBER(E11),ISNUMBER(G11)),G11-E11,"")</f>
+        <v/>
+      </c>
+      <c r="K11" s="18">
+        <f>IF(AND(ISNUMBER(G11),ISNUMBER(I11)),I11-G11,"")</f>
+        <v/>
+      </c>
+      <c r="L11" s="19">
+        <f>IF(AND(ISNUMBER(J11),ISNUMBER(K11)),IF(J11&gt;0,(J11+K11)/J11,""),"")</f>
+        <v/>
+      </c>
+      <c r="M11" s="5" t="n"/>
+      <c r="N11" s="5" t="n"/>
+      <c r="O11" s="3" t="inlineStr">
+        <is>
           <t>n/a: by difference</t>
         </is>
       </c>
-      <c r="P10" s="18" t="n"/>
-    </row>
-    <row r="11">
-      <c r="A11" s="11" t="inlineStr">
-        <is>
-          <t>BIN2</t>
-        </is>
-      </c>
-      <c r="B11" s="11" t="inlineStr">
-        <is>
-          <t>BIN2-B1</t>
-        </is>
-      </c>
-      <c r="C11" s="11" t="inlineStr">
-        <is>
-          <t>Inferior</t>
-        </is>
-      </c>
-      <c r="D11" s="11" t="inlineStr">
-        <is>
-          <t>aqueous</t>
-        </is>
-      </c>
-      <c r="E11" s="12" t="n"/>
-      <c r="F11" s="13" t="n">
-        <v>300</v>
-      </c>
-      <c r="G11" s="12" t="n"/>
-      <c r="H11" s="11">
-        <f>1000-F11</f>
-        <v/>
-      </c>
-      <c r="I11" s="12" t="n"/>
-      <c r="J11" s="14">
-        <f>IF(AND(ISNUMBER(E11),ISNUMBER(G11)),G11-E11,"")</f>
-        <v/>
-      </c>
-      <c r="K11" s="14">
-        <f>IF(AND(ISNUMBER(G11),ISNUMBER(I11)),I11-G11,"")</f>
-        <v/>
-      </c>
-      <c r="L11" s="15">
-        <f>IF(AND(ISNUMBER(J11),ISNUMBER(K11)),IF(J11&gt;0,(J11+K11)/J11,""),"")</f>
-        <v/>
-      </c>
-      <c r="M11" s="16" t="n"/>
-      <c r="N11" s="16" t="n"/>
-      <c r="O11" s="11" t="inlineStr">
-        <is>
-          <t>n/a: by difference</t>
-        </is>
-      </c>
-      <c r="P11" s="13" t="n"/>
+      <c r="P11" s="17" t="n"/>
     </row>
     <row r="12">
       <c r="A12" s="3" t="inlineStr">
         <is>
-          <t>BIN2</t>
+          <t>B5</t>
         </is>
       </c>
       <c r="B12" s="3" t="inlineStr">
         <is>
-          <t>BIN2-B2</t>
+          <t>B5-B2</t>
         </is>
       </c>
       <c r="C12" s="3" t="inlineStr">
@@ -996,25 +1025,25 @@
           <t>aqueous</t>
         </is>
       </c>
-      <c r="E12" s="17" t="n"/>
-      <c r="F12" s="18" t="n">
+      <c r="E12" s="16" t="n"/>
+      <c r="F12" s="17" t="n">
         <v>300</v>
       </c>
-      <c r="G12" s="17" t="n"/>
+      <c r="G12" s="16" t="n"/>
       <c r="H12" s="3">
         <f>1000-F12</f>
         <v/>
       </c>
-      <c r="I12" s="17" t="n"/>
-      <c r="J12" s="19">
+      <c r="I12" s="16" t="n"/>
+      <c r="J12" s="18">
         <f>IF(AND(ISNUMBER(E12),ISNUMBER(G12)),G12-E12,"")</f>
         <v/>
       </c>
-      <c r="K12" s="19">
+      <c r="K12" s="18">
         <f>IF(AND(ISNUMBER(G12),ISNUMBER(I12)),I12-G12,"")</f>
         <v/>
       </c>
-      <c r="L12" s="20">
+      <c r="L12" s="19">
         <f>IF(AND(ISNUMBER(J12),ISNUMBER(K12)),IF(J12&gt;0,(J12+K12)/J12,""),"")</f>
         <v/>
       </c>
@@ -1025,17 +1054,230 @@
           <t>n/a: by difference</t>
         </is>
       </c>
-      <c r="P12" s="18" t="n"/>
+      <c r="P12" s="17" t="n"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="11" t="inlineStr">
+        <is>
+          <t>BIN2</t>
+        </is>
+      </c>
+      <c r="B13" s="11" t="inlineStr">
+        <is>
+          <t>BIN2-T1</t>
+        </is>
+      </c>
+      <c r="C13" s="11" t="inlineStr">
+        <is>
+          <t>Superior</t>
+        </is>
+      </c>
+      <c r="D13" s="11" t="inlineStr">
+        <is>
+          <t>organic</t>
+        </is>
+      </c>
+      <c r="E13" s="12" t="n"/>
+      <c r="F13" s="13" t="n">
+        <v>300</v>
+      </c>
+      <c r="G13" s="12" t="n"/>
+      <c r="H13" s="11">
+        <f>1000-F13</f>
+        <v/>
+      </c>
+      <c r="I13" s="12" t="n"/>
+      <c r="J13" s="14">
+        <f>IF(AND(ISNUMBER(E13),ISNUMBER(G13)),G13-E13,"")</f>
+        <v/>
+      </c>
+      <c r="K13" s="14">
+        <f>IF(AND(ISNUMBER(G13),ISNUMBER(I13)),I13-G13,"")</f>
+        <v/>
+      </c>
+      <c r="L13" s="15">
+        <f>IF(AND(ISNUMBER(J13),ISNUMBER(K13)),IF(J13&gt;0,(J13+K13)/J13,""),"")</f>
+        <v/>
+      </c>
+      <c r="M13" s="13" t="n"/>
+      <c r="N13" s="13" t="n"/>
+      <c r="O13" s="11" t="inlineStr">
+        <is>
+          <t>fresh: type the new KF</t>
+        </is>
+      </c>
+      <c r="P13" s="13" t="n"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="3" t="inlineStr">
+        <is>
+          <t>BIN2</t>
+        </is>
+      </c>
+      <c r="B14" s="3" t="inlineStr">
+        <is>
+          <t>BIN2-T2</t>
+        </is>
+      </c>
+      <c r="C14" s="3" t="inlineStr">
+        <is>
+          <t>Superior</t>
+        </is>
+      </c>
+      <c r="D14" s="3" t="inlineStr">
+        <is>
+          <t>organic</t>
+        </is>
+      </c>
+      <c r="E14" s="16" t="n"/>
+      <c r="F14" s="17" t="n">
+        <v>300</v>
+      </c>
+      <c r="G14" s="16" t="n"/>
+      <c r="H14" s="3">
+        <f>1000-F14</f>
+        <v/>
+      </c>
+      <c r="I14" s="16" t="n"/>
+      <c r="J14" s="18">
+        <f>IF(AND(ISNUMBER(E14),ISNUMBER(G14)),G14-E14,"")</f>
+        <v/>
+      </c>
+      <c r="K14" s="18">
+        <f>IF(AND(ISNUMBER(G14),ISNUMBER(I14)),I14-G14,"")</f>
+        <v/>
+      </c>
+      <c r="L14" s="19">
+        <f>IF(AND(ISNUMBER(J14),ISNUMBER(K14)),IF(J14&gt;0,(J14+K14)/J14,""),"")</f>
+        <v/>
+      </c>
+      <c r="M14" s="17" t="n"/>
+      <c r="N14" s="17" t="n"/>
+      <c r="O14" s="3" t="inlineStr">
+        <is>
+          <t>fresh: type the new KF</t>
+        </is>
+      </c>
+      <c r="P14" s="17" t="n"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="3" t="inlineStr">
+        <is>
+          <t>BIN2</t>
+        </is>
+      </c>
+      <c r="B15" s="3" t="inlineStr">
+        <is>
+          <t>BIN2-B1</t>
+        </is>
+      </c>
+      <c r="C15" s="3" t="inlineStr">
+        <is>
+          <t>Inferior</t>
+        </is>
+      </c>
+      <c r="D15" s="3" t="inlineStr">
+        <is>
+          <t>aqueous</t>
+        </is>
+      </c>
+      <c r="E15" s="16" t="n"/>
+      <c r="F15" s="17" t="n">
+        <v>300</v>
+      </c>
+      <c r="G15" s="16" t="n"/>
+      <c r="H15" s="3">
+        <f>1000-F15</f>
+        <v/>
+      </c>
+      <c r="I15" s="16" t="n"/>
+      <c r="J15" s="18">
+        <f>IF(AND(ISNUMBER(E15),ISNUMBER(G15)),G15-E15,"")</f>
+        <v/>
+      </c>
+      <c r="K15" s="18">
+        <f>IF(AND(ISNUMBER(G15),ISNUMBER(I15)),I15-G15,"")</f>
+        <v/>
+      </c>
+      <c r="L15" s="19">
+        <f>IF(AND(ISNUMBER(J15),ISNUMBER(K15)),IF(J15&gt;0,(J15+K15)/J15,""),"")</f>
+        <v/>
+      </c>
+      <c r="M15" s="5" t="n"/>
+      <c r="N15" s="5" t="n"/>
+      <c r="O15" s="3" t="inlineStr">
+        <is>
+          <t>n/a: by difference</t>
+        </is>
+      </c>
+      <c r="P15" s="17" t="n"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="3" t="inlineStr">
+        <is>
+          <t>BIN2</t>
+        </is>
+      </c>
+      <c r="B16" s="3" t="inlineStr">
+        <is>
+          <t>BIN2-B2</t>
+        </is>
+      </c>
+      <c r="C16" s="3" t="inlineStr">
+        <is>
+          <t>Inferior</t>
+        </is>
+      </c>
+      <c r="D16" s="3" t="inlineStr">
+        <is>
+          <t>aqueous</t>
+        </is>
+      </c>
+      <c r="E16" s="16" t="n"/>
+      <c r="F16" s="17" t="n">
+        <v>300</v>
+      </c>
+      <c r="G16" s="16" t="n"/>
+      <c r="H16" s="3">
+        <f>1000-F16</f>
+        <v/>
+      </c>
+      <c r="I16" s="16" t="n"/>
+      <c r="J16" s="18">
+        <f>IF(AND(ISNUMBER(E16),ISNUMBER(G16)),G16-E16,"")</f>
+        <v/>
+      </c>
+      <c r="K16" s="18">
+        <f>IF(AND(ISNUMBER(G16),ISNUMBER(I16)),I16-G16,"")</f>
+        <v/>
+      </c>
+      <c r="L16" s="19">
+        <f>IF(AND(ISNUMBER(J16),ISNUMBER(K16)),IF(J16&gt;0,(J16+K16)/J16,""),"")</f>
+        <v/>
+      </c>
+      <c r="M16" s="5" t="n"/>
+      <c r="N16" s="5" t="n"/>
+      <c r="O16" s="3" t="inlineStr">
+        <is>
+          <t>n/a: by difference</t>
+        </is>
+      </c>
+      <c r="P16" s="17" t="n"/>
     </row>
   </sheetData>
   <sheetProtection selectLockedCells="0" selectUnlockedCells="0" sheet="1" objects="0" insertRows="1" insertHyperlinks="1" autoFilter="1" scenarios="0" formatColumns="1" deleteColumns="1" insertColumns="1" pivotTables="1" deleteRows="1" formatCells="1" formatRows="1" sort="1"/>
-  <dataValidations count="1">
-    <dataValidation sqref="E9:G9 E10:G10 E11:G11 E12:G12 I9 I10 I11 I12" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="0" error="A number between 0 and 100" type="decimal">
+  <dataValidations count="2">
+    <dataValidation sqref="E9:G9 E10:G10 E11:G11 E12:G12 E13:G13 E14:G14 E15:G15 E16:G16 I9 I10 I11 I12 I13 I14 I15 I16" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="0" error="A number between 0 and 100" type="decimal">
+      <formula1>0</formula1>
+      <formula2>100</formula2>
+    </dataValidation>
+    <dataValidation sqref="M9:N9 M10:N10 M13:N13 M14:N14" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="0" error="A number between 0 and 100" type="decimal">
       <formula1>0</formula1>
       <formula2>100</formula2>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>
+  <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
feat(repeat): round 3 re-measures the water-2PE binary too
The user's call, for the sake of it: 2PE joins B5 and BIN2 on the round-3 entry sheet
(12 vials; organic = bottom, fresh KF, as ORGANIC_OVERRIDE). Not in the prep book,
which only knows DES tubes -- the binary is water + 2PE, prepared by hand as in round 1.
When round 3 lands its 2PE codes override round 1's in two_pe_endpoint's merge.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/out/repeat3_entry.xlsx
+++ b/out/repeat3_entry.xlsx
@@ -93,7 +93,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="20">
+  <cellXfs count="21">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -126,6 +126,7 @@
     </xf>
     <xf numFmtId="164" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="2" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -521,7 +522,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:P16"/>
+  <dimension ref="A1:P20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -1264,14 +1265,222 @@
       </c>
       <c r="P16" s="17" t="n"/>
     </row>
+    <row r="17">
+      <c r="A17" s="11" t="inlineStr">
+        <is>
+          <t>2PE</t>
+        </is>
+      </c>
+      <c r="B17" s="11" t="inlineStr">
+        <is>
+          <t>2PE-T1</t>
+        </is>
+      </c>
+      <c r="C17" s="11" t="inlineStr">
+        <is>
+          <t>Superior</t>
+        </is>
+      </c>
+      <c r="D17" s="11" t="inlineStr">
+        <is>
+          <t>aqueous</t>
+        </is>
+      </c>
+      <c r="E17" s="12" t="n"/>
+      <c r="F17" s="13" t="n">
+        <v>300</v>
+      </c>
+      <c r="G17" s="12" t="n"/>
+      <c r="H17" s="11">
+        <f>1000-F17</f>
+        <v/>
+      </c>
+      <c r="I17" s="12" t="n"/>
+      <c r="J17" s="14">
+        <f>IF(AND(ISNUMBER(E17),ISNUMBER(G17)),G17-E17,"")</f>
+        <v/>
+      </c>
+      <c r="K17" s="14">
+        <f>IF(AND(ISNUMBER(G17),ISNUMBER(I17)),I17-G17,"")</f>
+        <v/>
+      </c>
+      <c r="L17" s="15">
+        <f>IF(AND(ISNUMBER(J17),ISNUMBER(K17)),IF(J17&gt;0,(J17+K17)/J17,""),"")</f>
+        <v/>
+      </c>
+      <c r="M17" s="20" t="n"/>
+      <c r="N17" s="20" t="n"/>
+      <c r="O17" s="11" t="inlineStr">
+        <is>
+          <t>n/a: by difference</t>
+        </is>
+      </c>
+      <c r="P17" s="13" t="n"/>
+    </row>
+    <row r="18">
+      <c r="A18" s="3" t="inlineStr">
+        <is>
+          <t>2PE</t>
+        </is>
+      </c>
+      <c r="B18" s="3" t="inlineStr">
+        <is>
+          <t>2PE-T2</t>
+        </is>
+      </c>
+      <c r="C18" s="3" t="inlineStr">
+        <is>
+          <t>Superior</t>
+        </is>
+      </c>
+      <c r="D18" s="3" t="inlineStr">
+        <is>
+          <t>aqueous</t>
+        </is>
+      </c>
+      <c r="E18" s="16" t="n"/>
+      <c r="F18" s="17" t="n">
+        <v>300</v>
+      </c>
+      <c r="G18" s="16" t="n"/>
+      <c r="H18" s="3">
+        <f>1000-F18</f>
+        <v/>
+      </c>
+      <c r="I18" s="16" t="n"/>
+      <c r="J18" s="18">
+        <f>IF(AND(ISNUMBER(E18),ISNUMBER(G18)),G18-E18,"")</f>
+        <v/>
+      </c>
+      <c r="K18" s="18">
+        <f>IF(AND(ISNUMBER(G18),ISNUMBER(I18)),I18-G18,"")</f>
+        <v/>
+      </c>
+      <c r="L18" s="19">
+        <f>IF(AND(ISNUMBER(J18),ISNUMBER(K18)),IF(J18&gt;0,(J18+K18)/J18,""),"")</f>
+        <v/>
+      </c>
+      <c r="M18" s="5" t="n"/>
+      <c r="N18" s="5" t="n"/>
+      <c r="O18" s="3" t="inlineStr">
+        <is>
+          <t>n/a: by difference</t>
+        </is>
+      </c>
+      <c r="P18" s="17" t="n"/>
+    </row>
+    <row r="19">
+      <c r="A19" s="3" t="inlineStr">
+        <is>
+          <t>2PE</t>
+        </is>
+      </c>
+      <c r="B19" s="3" t="inlineStr">
+        <is>
+          <t>2PE-B1</t>
+        </is>
+      </c>
+      <c r="C19" s="3" t="inlineStr">
+        <is>
+          <t>Inferior</t>
+        </is>
+      </c>
+      <c r="D19" s="3" t="inlineStr">
+        <is>
+          <t>organic</t>
+        </is>
+      </c>
+      <c r="E19" s="16" t="n"/>
+      <c r="F19" s="17" t="n">
+        <v>300</v>
+      </c>
+      <c r="G19" s="16" t="n"/>
+      <c r="H19" s="3">
+        <f>1000-F19</f>
+        <v/>
+      </c>
+      <c r="I19" s="16" t="n"/>
+      <c r="J19" s="18">
+        <f>IF(AND(ISNUMBER(E19),ISNUMBER(G19)),G19-E19,"")</f>
+        <v/>
+      </c>
+      <c r="K19" s="18">
+        <f>IF(AND(ISNUMBER(G19),ISNUMBER(I19)),I19-G19,"")</f>
+        <v/>
+      </c>
+      <c r="L19" s="19">
+        <f>IF(AND(ISNUMBER(J19),ISNUMBER(K19)),IF(J19&gt;0,(J19+K19)/J19,""),"")</f>
+        <v/>
+      </c>
+      <c r="M19" s="17" t="n"/>
+      <c r="N19" s="17" t="n"/>
+      <c r="O19" s="3" t="inlineStr">
+        <is>
+          <t>fresh: type the new KF</t>
+        </is>
+      </c>
+      <c r="P19" s="17" t="n"/>
+    </row>
+    <row r="20">
+      <c r="A20" s="3" t="inlineStr">
+        <is>
+          <t>2PE</t>
+        </is>
+      </c>
+      <c r="B20" s="3" t="inlineStr">
+        <is>
+          <t>2PE-B2</t>
+        </is>
+      </c>
+      <c r="C20" s="3" t="inlineStr">
+        <is>
+          <t>Inferior</t>
+        </is>
+      </c>
+      <c r="D20" s="3" t="inlineStr">
+        <is>
+          <t>organic</t>
+        </is>
+      </c>
+      <c r="E20" s="16" t="n"/>
+      <c r="F20" s="17" t="n">
+        <v>300</v>
+      </c>
+      <c r="G20" s="16" t="n"/>
+      <c r="H20" s="3">
+        <f>1000-F20</f>
+        <v/>
+      </c>
+      <c r="I20" s="16" t="n"/>
+      <c r="J20" s="18">
+        <f>IF(AND(ISNUMBER(E20),ISNUMBER(G20)),G20-E20,"")</f>
+        <v/>
+      </c>
+      <c r="K20" s="18">
+        <f>IF(AND(ISNUMBER(G20),ISNUMBER(I20)),I20-G20,"")</f>
+        <v/>
+      </c>
+      <c r="L20" s="19">
+        <f>IF(AND(ISNUMBER(J20),ISNUMBER(K20)),IF(J20&gt;0,(J20+K20)/J20,""),"")</f>
+        <v/>
+      </c>
+      <c r="M20" s="17" t="n"/>
+      <c r="N20" s="17" t="n"/>
+      <c r="O20" s="3" t="inlineStr">
+        <is>
+          <t>fresh: type the new KF</t>
+        </is>
+      </c>
+      <c r="P20" s="17" t="n"/>
+    </row>
   </sheetData>
   <sheetProtection selectLockedCells="0" selectUnlockedCells="0" sheet="1" objects="0" insertRows="1" insertHyperlinks="1" autoFilter="1" scenarios="0" formatColumns="1" deleteColumns="1" insertColumns="1" pivotTables="1" deleteRows="1" formatCells="1" formatRows="1" sort="1"/>
   <dataValidations count="2">
-    <dataValidation sqref="E9:G9 E10:G10 E11:G11 E12:G12 E13:G13 E14:G14 E15:G15 E16:G16 I9 I10 I11 I12 I13 I14 I15 I16" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="0" error="A number between 0 and 100" type="decimal">
+    <dataValidation sqref="E9:G9 E10:G10 E11:G11 E12:G12 E13:G13 E14:G14 E15:G15 E16:G16 E17:G17 E18:G18 E19:G19 E20:G20 I9 I10 I11 I12 I13 I14 I15 I16 I17 I18 I19 I20" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="0" error="A number between 0 and 100" type="decimal">
       <formula1>0</formula1>
       <formula2>100</formula2>
     </dataValidation>
-    <dataValidation sqref="M9:N9 M10:N10 M13:N13 M14:N14" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="0" error="A number between 0 and 100" type="decimal">
+    <dataValidation sqref="M9:N9 M10:N10 M13:N13 M14:N14 M19:N19 M20:N20" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="0" error="A number between 0 and 100" type="decimal">
       <formula1>0</formula1>
       <formula2>100</formula2>
     </dataValidation>

</xml_diff>

<commit_message>
feat(repeat): droplet pairs keep their leaner vial; round 3 adds F3 F4 H5 I4 BIN5 aqueous
aqueous_keep rule (3): below the saturation ceiling, an aqueous pair that fails the
replicate screen on component spread, with the terpenes the ones that moved, took organic
droplets into one vial -- carryover only adds, so the leaner vial is kept (A2, B1, B5, H2).
A 2PE-only disagreement stays flagged. An organic phase's whole-vial slip no longer flags
the point (mismatch_flag): it cancels in the KF anchor; transfer_factors still skips it.
The repeat list is now F3 F4 H5 I4 aqueous, the E edge and the B edge, and round 3's entry
sheet carries them: B5 BIN2 2PE whole plus F3:aq F4:aq H5:aq I4:aq BIN5:aq, 22 vials.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/out/repeat3_entry.xlsx
+++ b/out/repeat3_entry.xlsx
@@ -522,7 +522,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:P20"/>
+  <dimension ref="A1:P30"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -1268,17 +1268,17 @@
     <row r="17">
       <c r="A17" s="11" t="inlineStr">
         <is>
-          <t>2PE</t>
+          <t>BIN5</t>
         </is>
       </c>
       <c r="B17" s="11" t="inlineStr">
         <is>
-          <t>2PE-T1</t>
+          <t>BIN5-B1</t>
         </is>
       </c>
       <c r="C17" s="11" t="inlineStr">
         <is>
-          <t>Superior</t>
+          <t>Inferior</t>
         </is>
       </c>
       <c r="D17" s="11" t="inlineStr">
@@ -1320,17 +1320,17 @@
     <row r="18">
       <c r="A18" s="3" t="inlineStr">
         <is>
-          <t>2PE</t>
+          <t>BIN5</t>
         </is>
       </c>
       <c r="B18" s="3" t="inlineStr">
         <is>
-          <t>2PE-T2</t>
+          <t>BIN5-B2</t>
         </is>
       </c>
       <c r="C18" s="3" t="inlineStr">
         <is>
-          <t>Superior</t>
+          <t>Inferior</t>
         </is>
       </c>
       <c r="D18" s="3" t="inlineStr">
@@ -1370,66 +1370,66 @@
       <c r="P18" s="17" t="n"/>
     </row>
     <row r="19">
-      <c r="A19" s="3" t="inlineStr">
-        <is>
-          <t>2PE</t>
-        </is>
-      </c>
-      <c r="B19" s="3" t="inlineStr">
-        <is>
-          <t>2PE-B1</t>
-        </is>
-      </c>
-      <c r="C19" s="3" t="inlineStr">
+      <c r="A19" s="11" t="inlineStr">
+        <is>
+          <t>F3</t>
+        </is>
+      </c>
+      <c r="B19" s="11" t="inlineStr">
+        <is>
+          <t>F3-B1</t>
+        </is>
+      </c>
+      <c r="C19" s="11" t="inlineStr">
         <is>
           <t>Inferior</t>
         </is>
       </c>
-      <c r="D19" s="3" t="inlineStr">
-        <is>
-          <t>organic</t>
-        </is>
-      </c>
-      <c r="E19" s="16" t="n"/>
-      <c r="F19" s="17" t="n">
-        <v>300</v>
-      </c>
-      <c r="G19" s="16" t="n"/>
-      <c r="H19" s="3">
+      <c r="D19" s="11" t="inlineStr">
+        <is>
+          <t>aqueous</t>
+        </is>
+      </c>
+      <c r="E19" s="12" t="n"/>
+      <c r="F19" s="13" t="n">
+        <v>300</v>
+      </c>
+      <c r="G19" s="12" t="n"/>
+      <c r="H19" s="11">
         <f>1000-F19</f>
         <v/>
       </c>
-      <c r="I19" s="16" t="n"/>
-      <c r="J19" s="18">
+      <c r="I19" s="12" t="n"/>
+      <c r="J19" s="14">
         <f>IF(AND(ISNUMBER(E19),ISNUMBER(G19)),G19-E19,"")</f>
         <v/>
       </c>
-      <c r="K19" s="18">
+      <c r="K19" s="14">
         <f>IF(AND(ISNUMBER(G19),ISNUMBER(I19)),I19-G19,"")</f>
         <v/>
       </c>
-      <c r="L19" s="19">
+      <c r="L19" s="15">
         <f>IF(AND(ISNUMBER(J19),ISNUMBER(K19)),IF(J19&gt;0,(J19+K19)/J19,""),"")</f>
         <v/>
       </c>
-      <c r="M19" s="17" t="n"/>
-      <c r="N19" s="17" t="n"/>
-      <c r="O19" s="3" t="inlineStr">
-        <is>
-          <t>fresh: type the new KF</t>
-        </is>
-      </c>
-      <c r="P19" s="17" t="n"/>
+      <c r="M19" s="20" t="n"/>
+      <c r="N19" s="20" t="n"/>
+      <c r="O19" s="11" t="inlineStr">
+        <is>
+          <t>n/a: by difference</t>
+        </is>
+      </c>
+      <c r="P19" s="13" t="n"/>
     </row>
     <row r="20">
       <c r="A20" s="3" t="inlineStr">
         <is>
-          <t>2PE</t>
+          <t>F3</t>
         </is>
       </c>
       <c r="B20" s="3" t="inlineStr">
         <is>
-          <t>2PE-B2</t>
+          <t>F3-B2</t>
         </is>
       </c>
       <c r="C20" s="3" t="inlineStr">
@@ -1439,7 +1439,7 @@
       </c>
       <c r="D20" s="3" t="inlineStr">
         <is>
-          <t>organic</t>
+          <t>aqueous</t>
         </is>
       </c>
       <c r="E20" s="16" t="n"/>
@@ -1464,23 +1464,543 @@
         <f>IF(AND(ISNUMBER(J20),ISNUMBER(K20)),IF(J20&gt;0,(J20+K20)/J20,""),"")</f>
         <v/>
       </c>
-      <c r="M20" s="17" t="n"/>
-      <c r="N20" s="17" t="n"/>
+      <c r="M20" s="5" t="n"/>
+      <c r="N20" s="5" t="n"/>
       <c r="O20" s="3" t="inlineStr">
         <is>
+          <t>n/a: by difference</t>
+        </is>
+      </c>
+      <c r="P20" s="17" t="n"/>
+    </row>
+    <row r="21">
+      <c r="A21" s="11" t="inlineStr">
+        <is>
+          <t>F4</t>
+        </is>
+      </c>
+      <c r="B21" s="11" t="inlineStr">
+        <is>
+          <t>F4-B1</t>
+        </is>
+      </c>
+      <c r="C21" s="11" t="inlineStr">
+        <is>
+          <t>Inferior</t>
+        </is>
+      </c>
+      <c r="D21" s="11" t="inlineStr">
+        <is>
+          <t>aqueous</t>
+        </is>
+      </c>
+      <c r="E21" s="12" t="n"/>
+      <c r="F21" s="13" t="n">
+        <v>300</v>
+      </c>
+      <c r="G21" s="12" t="n"/>
+      <c r="H21" s="11">
+        <f>1000-F21</f>
+        <v/>
+      </c>
+      <c r="I21" s="12" t="n"/>
+      <c r="J21" s="14">
+        <f>IF(AND(ISNUMBER(E21),ISNUMBER(G21)),G21-E21,"")</f>
+        <v/>
+      </c>
+      <c r="K21" s="14">
+        <f>IF(AND(ISNUMBER(G21),ISNUMBER(I21)),I21-G21,"")</f>
+        <v/>
+      </c>
+      <c r="L21" s="15">
+        <f>IF(AND(ISNUMBER(J21),ISNUMBER(K21)),IF(J21&gt;0,(J21+K21)/J21,""),"")</f>
+        <v/>
+      </c>
+      <c r="M21" s="20" t="n"/>
+      <c r="N21" s="20" t="n"/>
+      <c r="O21" s="11" t="inlineStr">
+        <is>
+          <t>n/a: by difference</t>
+        </is>
+      </c>
+      <c r="P21" s="13" t="n"/>
+    </row>
+    <row r="22">
+      <c r="A22" s="3" t="inlineStr">
+        <is>
+          <t>F4</t>
+        </is>
+      </c>
+      <c r="B22" s="3" t="inlineStr">
+        <is>
+          <t>F4-B2</t>
+        </is>
+      </c>
+      <c r="C22" s="3" t="inlineStr">
+        <is>
+          <t>Inferior</t>
+        </is>
+      </c>
+      <c r="D22" s="3" t="inlineStr">
+        <is>
+          <t>aqueous</t>
+        </is>
+      </c>
+      <c r="E22" s="16" t="n"/>
+      <c r="F22" s="17" t="n">
+        <v>300</v>
+      </c>
+      <c r="G22" s="16" t="n"/>
+      <c r="H22" s="3">
+        <f>1000-F22</f>
+        <v/>
+      </c>
+      <c r="I22" s="16" t="n"/>
+      <c r="J22" s="18">
+        <f>IF(AND(ISNUMBER(E22),ISNUMBER(G22)),G22-E22,"")</f>
+        <v/>
+      </c>
+      <c r="K22" s="18">
+        <f>IF(AND(ISNUMBER(G22),ISNUMBER(I22)),I22-G22,"")</f>
+        <v/>
+      </c>
+      <c r="L22" s="19">
+        <f>IF(AND(ISNUMBER(J22),ISNUMBER(K22)),IF(J22&gt;0,(J22+K22)/J22,""),"")</f>
+        <v/>
+      </c>
+      <c r="M22" s="5" t="n"/>
+      <c r="N22" s="5" t="n"/>
+      <c r="O22" s="3" t="inlineStr">
+        <is>
+          <t>n/a: by difference</t>
+        </is>
+      </c>
+      <c r="P22" s="17" t="n"/>
+    </row>
+    <row r="23">
+      <c r="A23" s="11" t="inlineStr">
+        <is>
+          <t>H5</t>
+        </is>
+      </c>
+      <c r="B23" s="11" t="inlineStr">
+        <is>
+          <t>H5-B1</t>
+        </is>
+      </c>
+      <c r="C23" s="11" t="inlineStr">
+        <is>
+          <t>Inferior</t>
+        </is>
+      </c>
+      <c r="D23" s="11" t="inlineStr">
+        <is>
+          <t>aqueous</t>
+        </is>
+      </c>
+      <c r="E23" s="12" t="n"/>
+      <c r="F23" s="13" t="n">
+        <v>300</v>
+      </c>
+      <c r="G23" s="12" t="n"/>
+      <c r="H23" s="11">
+        <f>1000-F23</f>
+        <v/>
+      </c>
+      <c r="I23" s="12" t="n"/>
+      <c r="J23" s="14">
+        <f>IF(AND(ISNUMBER(E23),ISNUMBER(G23)),G23-E23,"")</f>
+        <v/>
+      </c>
+      <c r="K23" s="14">
+        <f>IF(AND(ISNUMBER(G23),ISNUMBER(I23)),I23-G23,"")</f>
+        <v/>
+      </c>
+      <c r="L23" s="15">
+        <f>IF(AND(ISNUMBER(J23),ISNUMBER(K23)),IF(J23&gt;0,(J23+K23)/J23,""),"")</f>
+        <v/>
+      </c>
+      <c r="M23" s="20" t="n"/>
+      <c r="N23" s="20" t="n"/>
+      <c r="O23" s="11" t="inlineStr">
+        <is>
+          <t>n/a: by difference</t>
+        </is>
+      </c>
+      <c r="P23" s="13" t="n"/>
+    </row>
+    <row r="24">
+      <c r="A24" s="3" t="inlineStr">
+        <is>
+          <t>H5</t>
+        </is>
+      </c>
+      <c r="B24" s="3" t="inlineStr">
+        <is>
+          <t>H5-B2</t>
+        </is>
+      </c>
+      <c r="C24" s="3" t="inlineStr">
+        <is>
+          <t>Inferior</t>
+        </is>
+      </c>
+      <c r="D24" s="3" t="inlineStr">
+        <is>
+          <t>aqueous</t>
+        </is>
+      </c>
+      <c r="E24" s="16" t="n"/>
+      <c r="F24" s="17" t="n">
+        <v>300</v>
+      </c>
+      <c r="G24" s="16" t="n"/>
+      <c r="H24" s="3">
+        <f>1000-F24</f>
+        <v/>
+      </c>
+      <c r="I24" s="16" t="n"/>
+      <c r="J24" s="18">
+        <f>IF(AND(ISNUMBER(E24),ISNUMBER(G24)),G24-E24,"")</f>
+        <v/>
+      </c>
+      <c r="K24" s="18">
+        <f>IF(AND(ISNUMBER(G24),ISNUMBER(I24)),I24-G24,"")</f>
+        <v/>
+      </c>
+      <c r="L24" s="19">
+        <f>IF(AND(ISNUMBER(J24),ISNUMBER(K24)),IF(J24&gt;0,(J24+K24)/J24,""),"")</f>
+        <v/>
+      </c>
+      <c r="M24" s="5" t="n"/>
+      <c r="N24" s="5" t="n"/>
+      <c r="O24" s="3" t="inlineStr">
+        <is>
+          <t>n/a: by difference</t>
+        </is>
+      </c>
+      <c r="P24" s="17" t="n"/>
+    </row>
+    <row r="25">
+      <c r="A25" s="11" t="inlineStr">
+        <is>
+          <t>I4</t>
+        </is>
+      </c>
+      <c r="B25" s="11" t="inlineStr">
+        <is>
+          <t>I4-T1</t>
+        </is>
+      </c>
+      <c r="C25" s="11" t="inlineStr">
+        <is>
+          <t>Superior</t>
+        </is>
+      </c>
+      <c r="D25" s="11" t="inlineStr">
+        <is>
+          <t>aqueous</t>
+        </is>
+      </c>
+      <c r="E25" s="12" t="n"/>
+      <c r="F25" s="13" t="n">
+        <v>300</v>
+      </c>
+      <c r="G25" s="12" t="n"/>
+      <c r="H25" s="11">
+        <f>1000-F25</f>
+        <v/>
+      </c>
+      <c r="I25" s="12" t="n"/>
+      <c r="J25" s="14">
+        <f>IF(AND(ISNUMBER(E25),ISNUMBER(G25)),G25-E25,"")</f>
+        <v/>
+      </c>
+      <c r="K25" s="14">
+        <f>IF(AND(ISNUMBER(G25),ISNUMBER(I25)),I25-G25,"")</f>
+        <v/>
+      </c>
+      <c r="L25" s="15">
+        <f>IF(AND(ISNUMBER(J25),ISNUMBER(K25)),IF(J25&gt;0,(J25+K25)/J25,""),"")</f>
+        <v/>
+      </c>
+      <c r="M25" s="20" t="n"/>
+      <c r="N25" s="20" t="n"/>
+      <c r="O25" s="11" t="inlineStr">
+        <is>
+          <t>n/a: by difference</t>
+        </is>
+      </c>
+      <c r="P25" s="13" t="n"/>
+    </row>
+    <row r="26">
+      <c r="A26" s="3" t="inlineStr">
+        <is>
+          <t>I4</t>
+        </is>
+      </c>
+      <c r="B26" s="3" t="inlineStr">
+        <is>
+          <t>I4-T2</t>
+        </is>
+      </c>
+      <c r="C26" s="3" t="inlineStr">
+        <is>
+          <t>Superior</t>
+        </is>
+      </c>
+      <c r="D26" s="3" t="inlineStr">
+        <is>
+          <t>aqueous</t>
+        </is>
+      </c>
+      <c r="E26" s="16" t="n"/>
+      <c r="F26" s="17" t="n">
+        <v>300</v>
+      </c>
+      <c r="G26" s="16" t="n"/>
+      <c r="H26" s="3">
+        <f>1000-F26</f>
+        <v/>
+      </c>
+      <c r="I26" s="16" t="n"/>
+      <c r="J26" s="18">
+        <f>IF(AND(ISNUMBER(E26),ISNUMBER(G26)),G26-E26,"")</f>
+        <v/>
+      </c>
+      <c r="K26" s="18">
+        <f>IF(AND(ISNUMBER(G26),ISNUMBER(I26)),I26-G26,"")</f>
+        <v/>
+      </c>
+      <c r="L26" s="19">
+        <f>IF(AND(ISNUMBER(J26),ISNUMBER(K26)),IF(J26&gt;0,(J26+K26)/J26,""),"")</f>
+        <v/>
+      </c>
+      <c r="M26" s="5" t="n"/>
+      <c r="N26" s="5" t="n"/>
+      <c r="O26" s="3" t="inlineStr">
+        <is>
+          <t>n/a: by difference</t>
+        </is>
+      </c>
+      <c r="P26" s="17" t="n"/>
+    </row>
+    <row r="27">
+      <c r="A27" s="11" t="inlineStr">
+        <is>
+          <t>2PE</t>
+        </is>
+      </c>
+      <c r="B27" s="11" t="inlineStr">
+        <is>
+          <t>2PE-T1</t>
+        </is>
+      </c>
+      <c r="C27" s="11" t="inlineStr">
+        <is>
+          <t>Superior</t>
+        </is>
+      </c>
+      <c r="D27" s="11" t="inlineStr">
+        <is>
+          <t>aqueous</t>
+        </is>
+      </c>
+      <c r="E27" s="12" t="n"/>
+      <c r="F27" s="13" t="n">
+        <v>300</v>
+      </c>
+      <c r="G27" s="12" t="n"/>
+      <c r="H27" s="11">
+        <f>1000-F27</f>
+        <v/>
+      </c>
+      <c r="I27" s="12" t="n"/>
+      <c r="J27" s="14">
+        <f>IF(AND(ISNUMBER(E27),ISNUMBER(G27)),G27-E27,"")</f>
+        <v/>
+      </c>
+      <c r="K27" s="14">
+        <f>IF(AND(ISNUMBER(G27),ISNUMBER(I27)),I27-G27,"")</f>
+        <v/>
+      </c>
+      <c r="L27" s="15">
+        <f>IF(AND(ISNUMBER(J27),ISNUMBER(K27)),IF(J27&gt;0,(J27+K27)/J27,""),"")</f>
+        <v/>
+      </c>
+      <c r="M27" s="20" t="n"/>
+      <c r="N27" s="20" t="n"/>
+      <c r="O27" s="11" t="inlineStr">
+        <is>
+          <t>n/a: by difference</t>
+        </is>
+      </c>
+      <c r="P27" s="13" t="n"/>
+    </row>
+    <row r="28">
+      <c r="A28" s="3" t="inlineStr">
+        <is>
+          <t>2PE</t>
+        </is>
+      </c>
+      <c r="B28" s="3" t="inlineStr">
+        <is>
+          <t>2PE-T2</t>
+        </is>
+      </c>
+      <c r="C28" s="3" t="inlineStr">
+        <is>
+          <t>Superior</t>
+        </is>
+      </c>
+      <c r="D28" s="3" t="inlineStr">
+        <is>
+          <t>aqueous</t>
+        </is>
+      </c>
+      <c r="E28" s="16" t="n"/>
+      <c r="F28" s="17" t="n">
+        <v>300</v>
+      </c>
+      <c r="G28" s="16" t="n"/>
+      <c r="H28" s="3">
+        <f>1000-F28</f>
+        <v/>
+      </c>
+      <c r="I28" s="16" t="n"/>
+      <c r="J28" s="18">
+        <f>IF(AND(ISNUMBER(E28),ISNUMBER(G28)),G28-E28,"")</f>
+        <v/>
+      </c>
+      <c r="K28" s="18">
+        <f>IF(AND(ISNUMBER(G28),ISNUMBER(I28)),I28-G28,"")</f>
+        <v/>
+      </c>
+      <c r="L28" s="19">
+        <f>IF(AND(ISNUMBER(J28),ISNUMBER(K28)),IF(J28&gt;0,(J28+K28)/J28,""),"")</f>
+        <v/>
+      </c>
+      <c r="M28" s="5" t="n"/>
+      <c r="N28" s="5" t="n"/>
+      <c r="O28" s="3" t="inlineStr">
+        <is>
+          <t>n/a: by difference</t>
+        </is>
+      </c>
+      <c r="P28" s="17" t="n"/>
+    </row>
+    <row r="29">
+      <c r="A29" s="3" t="inlineStr">
+        <is>
+          <t>2PE</t>
+        </is>
+      </c>
+      <c r="B29" s="3" t="inlineStr">
+        <is>
+          <t>2PE-B1</t>
+        </is>
+      </c>
+      <c r="C29" s="3" t="inlineStr">
+        <is>
+          <t>Inferior</t>
+        </is>
+      </c>
+      <c r="D29" s="3" t="inlineStr">
+        <is>
+          <t>organic</t>
+        </is>
+      </c>
+      <c r="E29" s="16" t="n"/>
+      <c r="F29" s="17" t="n">
+        <v>300</v>
+      </c>
+      <c r="G29" s="16" t="n"/>
+      <c r="H29" s="3">
+        <f>1000-F29</f>
+        <v/>
+      </c>
+      <c r="I29" s="16" t="n"/>
+      <c r="J29" s="18">
+        <f>IF(AND(ISNUMBER(E29),ISNUMBER(G29)),G29-E29,"")</f>
+        <v/>
+      </c>
+      <c r="K29" s="18">
+        <f>IF(AND(ISNUMBER(G29),ISNUMBER(I29)),I29-G29,"")</f>
+        <v/>
+      </c>
+      <c r="L29" s="19">
+        <f>IF(AND(ISNUMBER(J29),ISNUMBER(K29)),IF(J29&gt;0,(J29+K29)/J29,""),"")</f>
+        <v/>
+      </c>
+      <c r="M29" s="17" t="n"/>
+      <c r="N29" s="17" t="n"/>
+      <c r="O29" s="3" t="inlineStr">
+        <is>
           <t>fresh: type the new KF</t>
         </is>
       </c>
-      <c r="P20" s="17" t="n"/>
+      <c r="P29" s="17" t="n"/>
+    </row>
+    <row r="30">
+      <c r="A30" s="3" t="inlineStr">
+        <is>
+          <t>2PE</t>
+        </is>
+      </c>
+      <c r="B30" s="3" t="inlineStr">
+        <is>
+          <t>2PE-B2</t>
+        </is>
+      </c>
+      <c r="C30" s="3" t="inlineStr">
+        <is>
+          <t>Inferior</t>
+        </is>
+      </c>
+      <c r="D30" s="3" t="inlineStr">
+        <is>
+          <t>organic</t>
+        </is>
+      </c>
+      <c r="E30" s="16" t="n"/>
+      <c r="F30" s="17" t="n">
+        <v>300</v>
+      </c>
+      <c r="G30" s="16" t="n"/>
+      <c r="H30" s="3">
+        <f>1000-F30</f>
+        <v/>
+      </c>
+      <c r="I30" s="16" t="n"/>
+      <c r="J30" s="18">
+        <f>IF(AND(ISNUMBER(E30),ISNUMBER(G30)),G30-E30,"")</f>
+        <v/>
+      </c>
+      <c r="K30" s="18">
+        <f>IF(AND(ISNUMBER(G30),ISNUMBER(I30)),I30-G30,"")</f>
+        <v/>
+      </c>
+      <c r="L30" s="19">
+        <f>IF(AND(ISNUMBER(J30),ISNUMBER(K30)),IF(J30&gt;0,(J30+K30)/J30,""),"")</f>
+        <v/>
+      </c>
+      <c r="M30" s="17" t="n"/>
+      <c r="N30" s="17" t="n"/>
+      <c r="O30" s="3" t="inlineStr">
+        <is>
+          <t>fresh: type the new KF</t>
+        </is>
+      </c>
+      <c r="P30" s="17" t="n"/>
     </row>
   </sheetData>
   <sheetProtection selectLockedCells="0" selectUnlockedCells="0" sheet="1" objects="0" insertRows="1" insertHyperlinks="1" autoFilter="1" scenarios="0" formatColumns="1" deleteColumns="1" insertColumns="1" pivotTables="1" deleteRows="1" formatCells="1" formatRows="1" sort="1"/>
   <dataValidations count="2">
-    <dataValidation sqref="E9:G9 E10:G10 E11:G11 E12:G12 E13:G13 E14:G14 E15:G15 E16:G16 E17:G17 E18:G18 E19:G19 E20:G20 I9 I10 I11 I12 I13 I14 I15 I16 I17 I18 I19 I20" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="0" error="A number between 0 and 100" type="decimal">
+    <dataValidation sqref="E9:G9 E10:G10 E11:G11 E12:G12 E13:G13 E14:G14 E15:G15 E16:G16 E17:G17 E18:G18 E19:G19 E20:G20 E21:G21 E22:G22 E23:G23 E24:G24 E25:G25 E26:G26 E27:G27 E28:G28 E29:G29 E30:G30 I9 I10 I11 I12 I13 I14 I15 I16 I17 I18 I19 I20 I21 I22 I23 I24 I25 I26 I27 I28 I29 I30" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="0" error="A number between 0 and 100" type="decimal">
       <formula1>0</formula1>
       <formula2>100</formula2>
     </dataValidation>
-    <dataValidation sqref="M9:N9 M10:N10 M13:N13 M14:N14 M19:N19 M20:N20" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="0" error="A number between 0 and 100" type="decimal">
+    <dataValidation sqref="M9:N9 M10:N10 M13:N13 M14:N14 M29:N29 M30:N30" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="0" error="A number between 0 and 100" type="decimal">
       <formula1>0</formula1>
       <formula2>100</formula2>
     </dataValidation>

</xml_diff>

<commit_message>
feat(repeat): round 4 for this week's aqueous repeats; round 2 borrows round 1's phi
Round 3 (B5, BIN2, 2PE) was measured on 2026-09-28, so the tubes d074140 had added to it
move to a round of their own -- one round, one GC batch: round 4 = F3 F4 H2 H5 I4 BIN5,
aqueous only, 12 vials (H2's one surviving vial sits off both its block's terpene trend
and K). Round 3's entry sheet is back to its 28 Sep contents.

TRANSFER_PROXY: round 2 has no clean organic endpoint; it ran four days after round 1 on
the same method (2PE t_R 10.71 vs 10.70 min), so it borrows round 1's phi = 0.996 (the
user's call). TESIS carries the gap in the uncertainty.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/out/repeat3_entry.xlsx
+++ b/out/repeat3_entry.xlsx
@@ -522,7 +522,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:P30"/>
+  <dimension ref="A1:P20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -1268,17 +1268,17 @@
     <row r="17">
       <c r="A17" s="11" t="inlineStr">
         <is>
-          <t>BIN5</t>
+          <t>2PE</t>
         </is>
       </c>
       <c r="B17" s="11" t="inlineStr">
         <is>
-          <t>BIN5-B1</t>
+          <t>2PE-T1</t>
         </is>
       </c>
       <c r="C17" s="11" t="inlineStr">
         <is>
-          <t>Inferior</t>
+          <t>Superior</t>
         </is>
       </c>
       <c r="D17" s="11" t="inlineStr">
@@ -1320,17 +1320,17 @@
     <row r="18">
       <c r="A18" s="3" t="inlineStr">
         <is>
-          <t>BIN5</t>
+          <t>2PE</t>
         </is>
       </c>
       <c r="B18" s="3" t="inlineStr">
         <is>
-          <t>BIN5-B2</t>
+          <t>2PE-T2</t>
         </is>
       </c>
       <c r="C18" s="3" t="inlineStr">
         <is>
-          <t>Inferior</t>
+          <t>Superior</t>
         </is>
       </c>
       <c r="D18" s="3" t="inlineStr">
@@ -1370,66 +1370,66 @@
       <c r="P18" s="17" t="n"/>
     </row>
     <row r="19">
-      <c r="A19" s="11" t="inlineStr">
-        <is>
-          <t>F3</t>
-        </is>
-      </c>
-      <c r="B19" s="11" t="inlineStr">
-        <is>
-          <t>F3-B1</t>
-        </is>
-      </c>
-      <c r="C19" s="11" t="inlineStr">
+      <c r="A19" s="3" t="inlineStr">
+        <is>
+          <t>2PE</t>
+        </is>
+      </c>
+      <c r="B19" s="3" t="inlineStr">
+        <is>
+          <t>2PE-B1</t>
+        </is>
+      </c>
+      <c r="C19" s="3" t="inlineStr">
         <is>
           <t>Inferior</t>
         </is>
       </c>
-      <c r="D19" s="11" t="inlineStr">
-        <is>
-          <t>aqueous</t>
-        </is>
-      </c>
-      <c r="E19" s="12" t="n"/>
-      <c r="F19" s="13" t="n">
+      <c r="D19" s="3" t="inlineStr">
+        <is>
+          <t>organic</t>
+        </is>
+      </c>
+      <c r="E19" s="16" t="n"/>
+      <c r="F19" s="17" t="n">
         <v>300</v>
       </c>
-      <c r="G19" s="12" t="n"/>
-      <c r="H19" s="11">
+      <c r="G19" s="16" t="n"/>
+      <c r="H19" s="3">
         <f>1000-F19</f>
         <v/>
       </c>
-      <c r="I19" s="12" t="n"/>
-      <c r="J19" s="14">
+      <c r="I19" s="16" t="n"/>
+      <c r="J19" s="18">
         <f>IF(AND(ISNUMBER(E19),ISNUMBER(G19)),G19-E19,"")</f>
         <v/>
       </c>
-      <c r="K19" s="14">
+      <c r="K19" s="18">
         <f>IF(AND(ISNUMBER(G19),ISNUMBER(I19)),I19-G19,"")</f>
         <v/>
       </c>
-      <c r="L19" s="15">
+      <c r="L19" s="19">
         <f>IF(AND(ISNUMBER(J19),ISNUMBER(K19)),IF(J19&gt;0,(J19+K19)/J19,""),"")</f>
         <v/>
       </c>
-      <c r="M19" s="20" t="n"/>
-      <c r="N19" s="20" t="n"/>
-      <c r="O19" s="11" t="inlineStr">
-        <is>
-          <t>n/a: by difference</t>
-        </is>
-      </c>
-      <c r="P19" s="13" t="n"/>
+      <c r="M19" s="17" t="n"/>
+      <c r="N19" s="17" t="n"/>
+      <c r="O19" s="3" t="inlineStr">
+        <is>
+          <t>fresh: type the new KF</t>
+        </is>
+      </c>
+      <c r="P19" s="17" t="n"/>
     </row>
     <row r="20">
       <c r="A20" s="3" t="inlineStr">
         <is>
-          <t>F3</t>
+          <t>2PE</t>
         </is>
       </c>
       <c r="B20" s="3" t="inlineStr">
         <is>
-          <t>F3-B2</t>
+          <t>2PE-B2</t>
         </is>
       </c>
       <c r="C20" s="3" t="inlineStr">
@@ -1439,7 +1439,7 @@
       </c>
       <c r="D20" s="3" t="inlineStr">
         <is>
-          <t>aqueous</t>
+          <t>organic</t>
         </is>
       </c>
       <c r="E20" s="16" t="n"/>
@@ -1464,543 +1464,23 @@
         <f>IF(AND(ISNUMBER(J20),ISNUMBER(K20)),IF(J20&gt;0,(J20+K20)/J20,""),"")</f>
         <v/>
       </c>
-      <c r="M20" s="5" t="n"/>
-      <c r="N20" s="5" t="n"/>
+      <c r="M20" s="17" t="n"/>
+      <c r="N20" s="17" t="n"/>
       <c r="O20" s="3" t="inlineStr">
         <is>
-          <t>n/a: by difference</t>
+          <t>fresh: type the new KF</t>
         </is>
       </c>
       <c r="P20" s="17" t="n"/>
-    </row>
-    <row r="21">
-      <c r="A21" s="11" t="inlineStr">
-        <is>
-          <t>F4</t>
-        </is>
-      </c>
-      <c r="B21" s="11" t="inlineStr">
-        <is>
-          <t>F4-B1</t>
-        </is>
-      </c>
-      <c r="C21" s="11" t="inlineStr">
-        <is>
-          <t>Inferior</t>
-        </is>
-      </c>
-      <c r="D21" s="11" t="inlineStr">
-        <is>
-          <t>aqueous</t>
-        </is>
-      </c>
-      <c r="E21" s="12" t="n"/>
-      <c r="F21" s="13" t="n">
-        <v>300</v>
-      </c>
-      <c r="G21" s="12" t="n"/>
-      <c r="H21" s="11">
-        <f>1000-F21</f>
-        <v/>
-      </c>
-      <c r="I21" s="12" t="n"/>
-      <c r="J21" s="14">
-        <f>IF(AND(ISNUMBER(E21),ISNUMBER(G21)),G21-E21,"")</f>
-        <v/>
-      </c>
-      <c r="K21" s="14">
-        <f>IF(AND(ISNUMBER(G21),ISNUMBER(I21)),I21-G21,"")</f>
-        <v/>
-      </c>
-      <c r="L21" s="15">
-        <f>IF(AND(ISNUMBER(J21),ISNUMBER(K21)),IF(J21&gt;0,(J21+K21)/J21,""),"")</f>
-        <v/>
-      </c>
-      <c r="M21" s="20" t="n"/>
-      <c r="N21" s="20" t="n"/>
-      <c r="O21" s="11" t="inlineStr">
-        <is>
-          <t>n/a: by difference</t>
-        </is>
-      </c>
-      <c r="P21" s="13" t="n"/>
-    </row>
-    <row r="22">
-      <c r="A22" s="3" t="inlineStr">
-        <is>
-          <t>F4</t>
-        </is>
-      </c>
-      <c r="B22" s="3" t="inlineStr">
-        <is>
-          <t>F4-B2</t>
-        </is>
-      </c>
-      <c r="C22" s="3" t="inlineStr">
-        <is>
-          <t>Inferior</t>
-        </is>
-      </c>
-      <c r="D22" s="3" t="inlineStr">
-        <is>
-          <t>aqueous</t>
-        </is>
-      </c>
-      <c r="E22" s="16" t="n"/>
-      <c r="F22" s="17" t="n">
-        <v>300</v>
-      </c>
-      <c r="G22" s="16" t="n"/>
-      <c r="H22" s="3">
-        <f>1000-F22</f>
-        <v/>
-      </c>
-      <c r="I22" s="16" t="n"/>
-      <c r="J22" s="18">
-        <f>IF(AND(ISNUMBER(E22),ISNUMBER(G22)),G22-E22,"")</f>
-        <v/>
-      </c>
-      <c r="K22" s="18">
-        <f>IF(AND(ISNUMBER(G22),ISNUMBER(I22)),I22-G22,"")</f>
-        <v/>
-      </c>
-      <c r="L22" s="19">
-        <f>IF(AND(ISNUMBER(J22),ISNUMBER(K22)),IF(J22&gt;0,(J22+K22)/J22,""),"")</f>
-        <v/>
-      </c>
-      <c r="M22" s="5" t="n"/>
-      <c r="N22" s="5" t="n"/>
-      <c r="O22" s="3" t="inlineStr">
-        <is>
-          <t>n/a: by difference</t>
-        </is>
-      </c>
-      <c r="P22" s="17" t="n"/>
-    </row>
-    <row r="23">
-      <c r="A23" s="11" t="inlineStr">
-        <is>
-          <t>H5</t>
-        </is>
-      </c>
-      <c r="B23" s="11" t="inlineStr">
-        <is>
-          <t>H5-B1</t>
-        </is>
-      </c>
-      <c r="C23" s="11" t="inlineStr">
-        <is>
-          <t>Inferior</t>
-        </is>
-      </c>
-      <c r="D23" s="11" t="inlineStr">
-        <is>
-          <t>aqueous</t>
-        </is>
-      </c>
-      <c r="E23" s="12" t="n"/>
-      <c r="F23" s="13" t="n">
-        <v>300</v>
-      </c>
-      <c r="G23" s="12" t="n"/>
-      <c r="H23" s="11">
-        <f>1000-F23</f>
-        <v/>
-      </c>
-      <c r="I23" s="12" t="n"/>
-      <c r="J23" s="14">
-        <f>IF(AND(ISNUMBER(E23),ISNUMBER(G23)),G23-E23,"")</f>
-        <v/>
-      </c>
-      <c r="K23" s="14">
-        <f>IF(AND(ISNUMBER(G23),ISNUMBER(I23)),I23-G23,"")</f>
-        <v/>
-      </c>
-      <c r="L23" s="15">
-        <f>IF(AND(ISNUMBER(J23),ISNUMBER(K23)),IF(J23&gt;0,(J23+K23)/J23,""),"")</f>
-        <v/>
-      </c>
-      <c r="M23" s="20" t="n"/>
-      <c r="N23" s="20" t="n"/>
-      <c r="O23" s="11" t="inlineStr">
-        <is>
-          <t>n/a: by difference</t>
-        </is>
-      </c>
-      <c r="P23" s="13" t="n"/>
-    </row>
-    <row r="24">
-      <c r="A24" s="3" t="inlineStr">
-        <is>
-          <t>H5</t>
-        </is>
-      </c>
-      <c r="B24" s="3" t="inlineStr">
-        <is>
-          <t>H5-B2</t>
-        </is>
-      </c>
-      <c r="C24" s="3" t="inlineStr">
-        <is>
-          <t>Inferior</t>
-        </is>
-      </c>
-      <c r="D24" s="3" t="inlineStr">
-        <is>
-          <t>aqueous</t>
-        </is>
-      </c>
-      <c r="E24" s="16" t="n"/>
-      <c r="F24" s="17" t="n">
-        <v>300</v>
-      </c>
-      <c r="G24" s="16" t="n"/>
-      <c r="H24" s="3">
-        <f>1000-F24</f>
-        <v/>
-      </c>
-      <c r="I24" s="16" t="n"/>
-      <c r="J24" s="18">
-        <f>IF(AND(ISNUMBER(E24),ISNUMBER(G24)),G24-E24,"")</f>
-        <v/>
-      </c>
-      <c r="K24" s="18">
-        <f>IF(AND(ISNUMBER(G24),ISNUMBER(I24)),I24-G24,"")</f>
-        <v/>
-      </c>
-      <c r="L24" s="19">
-        <f>IF(AND(ISNUMBER(J24),ISNUMBER(K24)),IF(J24&gt;0,(J24+K24)/J24,""),"")</f>
-        <v/>
-      </c>
-      <c r="M24" s="5" t="n"/>
-      <c r="N24" s="5" t="n"/>
-      <c r="O24" s="3" t="inlineStr">
-        <is>
-          <t>n/a: by difference</t>
-        </is>
-      </c>
-      <c r="P24" s="17" t="n"/>
-    </row>
-    <row r="25">
-      <c r="A25" s="11" t="inlineStr">
-        <is>
-          <t>I4</t>
-        </is>
-      </c>
-      <c r="B25" s="11" t="inlineStr">
-        <is>
-          <t>I4-T1</t>
-        </is>
-      </c>
-      <c r="C25" s="11" t="inlineStr">
-        <is>
-          <t>Superior</t>
-        </is>
-      </c>
-      <c r="D25" s="11" t="inlineStr">
-        <is>
-          <t>aqueous</t>
-        </is>
-      </c>
-      <c r="E25" s="12" t="n"/>
-      <c r="F25" s="13" t="n">
-        <v>300</v>
-      </c>
-      <c r="G25" s="12" t="n"/>
-      <c r="H25" s="11">
-        <f>1000-F25</f>
-        <v/>
-      </c>
-      <c r="I25" s="12" t="n"/>
-      <c r="J25" s="14">
-        <f>IF(AND(ISNUMBER(E25),ISNUMBER(G25)),G25-E25,"")</f>
-        <v/>
-      </c>
-      <c r="K25" s="14">
-        <f>IF(AND(ISNUMBER(G25),ISNUMBER(I25)),I25-G25,"")</f>
-        <v/>
-      </c>
-      <c r="L25" s="15">
-        <f>IF(AND(ISNUMBER(J25),ISNUMBER(K25)),IF(J25&gt;0,(J25+K25)/J25,""),"")</f>
-        <v/>
-      </c>
-      <c r="M25" s="20" t="n"/>
-      <c r="N25" s="20" t="n"/>
-      <c r="O25" s="11" t="inlineStr">
-        <is>
-          <t>n/a: by difference</t>
-        </is>
-      </c>
-      <c r="P25" s="13" t="n"/>
-    </row>
-    <row r="26">
-      <c r="A26" s="3" t="inlineStr">
-        <is>
-          <t>I4</t>
-        </is>
-      </c>
-      <c r="B26" s="3" t="inlineStr">
-        <is>
-          <t>I4-T2</t>
-        </is>
-      </c>
-      <c r="C26" s="3" t="inlineStr">
-        <is>
-          <t>Superior</t>
-        </is>
-      </c>
-      <c r="D26" s="3" t="inlineStr">
-        <is>
-          <t>aqueous</t>
-        </is>
-      </c>
-      <c r="E26" s="16" t="n"/>
-      <c r="F26" s="17" t="n">
-        <v>300</v>
-      </c>
-      <c r="G26" s="16" t="n"/>
-      <c r="H26" s="3">
-        <f>1000-F26</f>
-        <v/>
-      </c>
-      <c r="I26" s="16" t="n"/>
-      <c r="J26" s="18">
-        <f>IF(AND(ISNUMBER(E26),ISNUMBER(G26)),G26-E26,"")</f>
-        <v/>
-      </c>
-      <c r="K26" s="18">
-        <f>IF(AND(ISNUMBER(G26),ISNUMBER(I26)),I26-G26,"")</f>
-        <v/>
-      </c>
-      <c r="L26" s="19">
-        <f>IF(AND(ISNUMBER(J26),ISNUMBER(K26)),IF(J26&gt;0,(J26+K26)/J26,""),"")</f>
-        <v/>
-      </c>
-      <c r="M26" s="5" t="n"/>
-      <c r="N26" s="5" t="n"/>
-      <c r="O26" s="3" t="inlineStr">
-        <is>
-          <t>n/a: by difference</t>
-        </is>
-      </c>
-      <c r="P26" s="17" t="n"/>
-    </row>
-    <row r="27">
-      <c r="A27" s="11" t="inlineStr">
-        <is>
-          <t>2PE</t>
-        </is>
-      </c>
-      <c r="B27" s="11" t="inlineStr">
-        <is>
-          <t>2PE-T1</t>
-        </is>
-      </c>
-      <c r="C27" s="11" t="inlineStr">
-        <is>
-          <t>Superior</t>
-        </is>
-      </c>
-      <c r="D27" s="11" t="inlineStr">
-        <is>
-          <t>aqueous</t>
-        </is>
-      </c>
-      <c r="E27" s="12" t="n"/>
-      <c r="F27" s="13" t="n">
-        <v>300</v>
-      </c>
-      <c r="G27" s="12" t="n"/>
-      <c r="H27" s="11">
-        <f>1000-F27</f>
-        <v/>
-      </c>
-      <c r="I27" s="12" t="n"/>
-      <c r="J27" s="14">
-        <f>IF(AND(ISNUMBER(E27),ISNUMBER(G27)),G27-E27,"")</f>
-        <v/>
-      </c>
-      <c r="K27" s="14">
-        <f>IF(AND(ISNUMBER(G27),ISNUMBER(I27)),I27-G27,"")</f>
-        <v/>
-      </c>
-      <c r="L27" s="15">
-        <f>IF(AND(ISNUMBER(J27),ISNUMBER(K27)),IF(J27&gt;0,(J27+K27)/J27,""),"")</f>
-        <v/>
-      </c>
-      <c r="M27" s="20" t="n"/>
-      <c r="N27" s="20" t="n"/>
-      <c r="O27" s="11" t="inlineStr">
-        <is>
-          <t>n/a: by difference</t>
-        </is>
-      </c>
-      <c r="P27" s="13" t="n"/>
-    </row>
-    <row r="28">
-      <c r="A28" s="3" t="inlineStr">
-        <is>
-          <t>2PE</t>
-        </is>
-      </c>
-      <c r="B28" s="3" t="inlineStr">
-        <is>
-          <t>2PE-T2</t>
-        </is>
-      </c>
-      <c r="C28" s="3" t="inlineStr">
-        <is>
-          <t>Superior</t>
-        </is>
-      </c>
-      <c r="D28" s="3" t="inlineStr">
-        <is>
-          <t>aqueous</t>
-        </is>
-      </c>
-      <c r="E28" s="16" t="n"/>
-      <c r="F28" s="17" t="n">
-        <v>300</v>
-      </c>
-      <c r="G28" s="16" t="n"/>
-      <c r="H28" s="3">
-        <f>1000-F28</f>
-        <v/>
-      </c>
-      <c r="I28" s="16" t="n"/>
-      <c r="J28" s="18">
-        <f>IF(AND(ISNUMBER(E28),ISNUMBER(G28)),G28-E28,"")</f>
-        <v/>
-      </c>
-      <c r="K28" s="18">
-        <f>IF(AND(ISNUMBER(G28),ISNUMBER(I28)),I28-G28,"")</f>
-        <v/>
-      </c>
-      <c r="L28" s="19">
-        <f>IF(AND(ISNUMBER(J28),ISNUMBER(K28)),IF(J28&gt;0,(J28+K28)/J28,""),"")</f>
-        <v/>
-      </c>
-      <c r="M28" s="5" t="n"/>
-      <c r="N28" s="5" t="n"/>
-      <c r="O28" s="3" t="inlineStr">
-        <is>
-          <t>n/a: by difference</t>
-        </is>
-      </c>
-      <c r="P28" s="17" t="n"/>
-    </row>
-    <row r="29">
-      <c r="A29" s="3" t="inlineStr">
-        <is>
-          <t>2PE</t>
-        </is>
-      </c>
-      <c r="B29" s="3" t="inlineStr">
-        <is>
-          <t>2PE-B1</t>
-        </is>
-      </c>
-      <c r="C29" s="3" t="inlineStr">
-        <is>
-          <t>Inferior</t>
-        </is>
-      </c>
-      <c r="D29" s="3" t="inlineStr">
-        <is>
-          <t>organic</t>
-        </is>
-      </c>
-      <c r="E29" s="16" t="n"/>
-      <c r="F29" s="17" t="n">
-        <v>300</v>
-      </c>
-      <c r="G29" s="16" t="n"/>
-      <c r="H29" s="3">
-        <f>1000-F29</f>
-        <v/>
-      </c>
-      <c r="I29" s="16" t="n"/>
-      <c r="J29" s="18">
-        <f>IF(AND(ISNUMBER(E29),ISNUMBER(G29)),G29-E29,"")</f>
-        <v/>
-      </c>
-      <c r="K29" s="18">
-        <f>IF(AND(ISNUMBER(G29),ISNUMBER(I29)),I29-G29,"")</f>
-        <v/>
-      </c>
-      <c r="L29" s="19">
-        <f>IF(AND(ISNUMBER(J29),ISNUMBER(K29)),IF(J29&gt;0,(J29+K29)/J29,""),"")</f>
-        <v/>
-      </c>
-      <c r="M29" s="17" t="n"/>
-      <c r="N29" s="17" t="n"/>
-      <c r="O29" s="3" t="inlineStr">
-        <is>
-          <t>fresh: type the new KF</t>
-        </is>
-      </c>
-      <c r="P29" s="17" t="n"/>
-    </row>
-    <row r="30">
-      <c r="A30" s="3" t="inlineStr">
-        <is>
-          <t>2PE</t>
-        </is>
-      </c>
-      <c r="B30" s="3" t="inlineStr">
-        <is>
-          <t>2PE-B2</t>
-        </is>
-      </c>
-      <c r="C30" s="3" t="inlineStr">
-        <is>
-          <t>Inferior</t>
-        </is>
-      </c>
-      <c r="D30" s="3" t="inlineStr">
-        <is>
-          <t>organic</t>
-        </is>
-      </c>
-      <c r="E30" s="16" t="n"/>
-      <c r="F30" s="17" t="n">
-        <v>300</v>
-      </c>
-      <c r="G30" s="16" t="n"/>
-      <c r="H30" s="3">
-        <f>1000-F30</f>
-        <v/>
-      </c>
-      <c r="I30" s="16" t="n"/>
-      <c r="J30" s="18">
-        <f>IF(AND(ISNUMBER(E30),ISNUMBER(G30)),G30-E30,"")</f>
-        <v/>
-      </c>
-      <c r="K30" s="18">
-        <f>IF(AND(ISNUMBER(G30),ISNUMBER(I30)),I30-G30,"")</f>
-        <v/>
-      </c>
-      <c r="L30" s="19">
-        <f>IF(AND(ISNUMBER(J30),ISNUMBER(K30)),IF(J30&gt;0,(J30+K30)/J30,""),"")</f>
-        <v/>
-      </c>
-      <c r="M30" s="17" t="n"/>
-      <c r="N30" s="17" t="n"/>
-      <c r="O30" s="3" t="inlineStr">
-        <is>
-          <t>fresh: type the new KF</t>
-        </is>
-      </c>
-      <c r="P30" s="17" t="n"/>
     </row>
   </sheetData>
   <sheetProtection selectLockedCells="0" selectUnlockedCells="0" sheet="1" objects="0" insertRows="1" insertHyperlinks="1" autoFilter="1" scenarios="0" formatColumns="1" deleteColumns="1" insertColumns="1" pivotTables="1" deleteRows="1" formatCells="1" formatRows="1" sort="1"/>
   <dataValidations count="2">
-    <dataValidation sqref="E9:G9 E10:G10 E11:G11 E12:G12 E13:G13 E14:G14 E15:G15 E16:G16 E17:G17 E18:G18 E19:G19 E20:G20 E21:G21 E22:G22 E23:G23 E24:G24 E25:G25 E26:G26 E27:G27 E28:G28 E29:G29 E30:G30 I9 I10 I11 I12 I13 I14 I15 I16 I17 I18 I19 I20 I21 I22 I23 I24 I25 I26 I27 I28 I29 I30" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="0" error="A number between 0 and 100" type="decimal">
+    <dataValidation sqref="E9:G9 E10:G10 E11:G11 E12:G12 E13:G13 E14:G14 E15:G15 E16:G16 E17:G17 E18:G18 E19:G19 E20:G20 I9 I10 I11 I12 I13 I14 I15 I16 I17 I18 I19 I20" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="0" error="A number between 0 and 100" type="decimal">
       <formula1>0</formula1>
       <formula2>100</formula2>
     </dataValidation>
-    <dataValidation sqref="M9:N9 M10:N10 M13:N13 M14:N14 M29:N29 M30:N30" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="0" error="A number between 0 and 100" type="decimal">
+    <dataValidation sqref="M9:N9 M10:N10 M13:N13 M14:N14 M19:N19 M20:N20" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="0" error="A number between 0 and 100" type="decimal">
       <formula1>0</formula1>
       <formula2>100</formula2>
     </dataValidation>

</xml_diff>